<commit_message>
All csv data after running R
All csv data after running R
</commit_message>
<xml_diff>
--- a/Code/Data/Groundtruth/Phylum.xlsx
+++ b/Code/Data/Groundtruth/Phylum.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AL-GHADIR\Desktop\Code\Data\Gund Truth\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AL-GHADIR\Desktop\Code\Data\Groundtruth\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E8E6A430-2855-479C-A0D3-DFB6C42C472B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{345603E2-C4F4-4EED-918B-31AC500A243B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{470BA22C-0DAD-48DE-B1B8-3AFDD5710E61}"/>
   </bookViews>
@@ -24,15 +24,25 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Consolas"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="2">
@@ -55,8 +65,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="2"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -371,33 +384,36 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{97C87C8C-CC14-4E85-B14C-936EA38480AA}">
-  <dimension ref="A1:A5"/>
+  <dimension ref="A1:A6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A1">
-        <v>-0.30030000000000001</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A2">
-        <v>0.247</v>
+        <v>-5</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A3">
-        <v>-0.2006</v>
+        <v>-0.65</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A4">
-        <v>-0.18290000000000001</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A5">
-        <v>-6.9199999999999998E-2</v>
+        <v>-7.8</v>
       </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A6" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>